<commit_message>
fix - Cập nhật lại địa chỉ công ty mới trên HĐ của NT1
</commit_message>
<xml_diff>
--- a/static/uploads/mau/hopdong/nt1/duoi_o2/hdcth.xlsx
+++ b/static/uploads/mau/hopdong/nt1/duoi_o2/hdcth.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DAT\Desktop\code\working\HRM\static\uploads\mau\hopdong\nt1\duoi_o2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DTD\Code\HRM\static\uploads\mau\hopdong\nt1\duoi_o2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A469781-DA81-4A60-BBB4-9F6F47E2BF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D21BDA50-EBE6-4804-BF52-9A618B907F97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MẪU IN HỢP ĐỒNG LAO ĐỘNG" sheetId="2" r:id="rId1"/>
@@ -487,14 +487,14 @@
     <t>của pháp luật về lao động và quy định của bảo hiểm	.</t>
   </si>
   <si>
-    <t>Địa chỉ: TDP 7 - Thuỷ Đường - Thuỷ Nguyên - Hải Phòng
+    <t>- Địa điểm làm việc: + Tổ dân phố 7, Phường Thủy Nguyên, TP Hải Phòng</t>
+  </si>
+  <si>
+    <t>Địa chỉ: TDP 7 - Thuỷ Nguyên - Hải Phòng
 ĐT: 02253.642.408</t>
   </si>
   <si>
-    <t>Tổ dân phố 7, Phường Thủy Đường, TP Thủy Nguyên, TP Hải Phòng</t>
-  </si>
-  <si>
-    <t>- Địa điểm làm việc: + Tổ dân phố 7, Phường Thủy Đường, TP Thủy Nguyên, TP Hải Phòng</t>
+    <t>Tổ dân phố 7, Phường Thủy Nguyên, TP Hải Phòng</t>
   </si>
 </sst>
 </file>
@@ -1140,7 +1140,7 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:X138"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="4" customWidth="1"/>
     <col min="9" max="10" width="8" customWidth="1"/>
@@ -1148,7 +1148,7 @@
     <col min="13" max="24" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16"/>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1178,13 +1178,13 @@
       <c r="W1" s="17"/>
       <c r="X1" s="17"/>
     </row>
-    <row r="2" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
       <c r="E2" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F2" s="19"/>
       <c r="G2" s="19"/>
@@ -1208,7 +1208,7 @@
       <c r="W2" s="20"/>
       <c r="X2" s="20"/>
     </row>
-    <row r="3" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1238,7 +1238,7 @@
       <c r="W3" s="20"/>
       <c r="X3" s="20"/>
     </row>
-    <row r="4" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1268,7 +1268,7 @@
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
     </row>
-    <row r="5" spans="1:24" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1294,7 +1294,7 @@
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
     </row>
-    <row r="6" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
         <v>6</v>
       </c>
@@ -1322,7 +1322,7 @@
       <c r="W6" s="21"/>
       <c r="X6" s="21"/>
     </row>
-    <row r="7" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
         <v>7</v>
       </c>
@@ -1350,7 +1350,7 @@
       <c r="W7" s="22"/>
       <c r="X7" s="22"/>
     </row>
-    <row r="8" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1376,7 +1376,7 @@
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
     </row>
-    <row r="9" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="8" t="s">
         <v>8</v>
@@ -1404,7 +1404,7 @@
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
     </row>
-    <row r="10" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="5" t="s">
         <v>9</v>
@@ -1438,7 +1438,7 @@
       <c r="W10" s="8"/>
       <c r="X10" s="8"/>
     </row>
-    <row r="11" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="5" t="s">
         <v>13</v>
@@ -1472,7 +1472,7 @@
       <c r="W11" s="5"/>
       <c r="X11" s="5"/>
     </row>
-    <row r="12" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="5" t="s">
         <v>17</v>
@@ -1502,7 +1502,7 @@
       <c r="W12" s="5"/>
       <c r="X12" s="5"/>
     </row>
-    <row r="13" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="5" t="s">
         <v>19</v>
@@ -1540,7 +1540,7 @@
       <c r="W13" s="5"/>
       <c r="X13" s="5"/>
     </row>
-    <row r="14" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="5" t="s">
         <v>25</v>
@@ -1570,14 +1570,14 @@
       <c r="W14" s="8"/>
       <c r="X14" s="8"/>
     </row>
-    <row r="15" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
@@ -1600,7 +1600,7 @@
       <c r="W15" s="5"/>
       <c r="X15" s="5"/>
     </row>
-    <row r="16" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="5" t="s">
         <v>27</v>
@@ -1634,7 +1634,7 @@
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
     </row>
-    <row r="17" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="8" t="s">
         <v>31</v>
@@ -1662,7 +1662,7 @@
       <c r="W17" s="2"/>
       <c r="X17" s="2"/>
     </row>
-    <row r="18" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="5" t="s">
         <v>9</v>
@@ -1696,7 +1696,7 @@
       <c r="W18" s="8"/>
       <c r="X18" s="8"/>
     </row>
-    <row r="19" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="5" t="s">
         <v>15</v>
@@ -1730,7 +1730,7 @@
       <c r="W19" s="5"/>
       <c r="X19" s="5"/>
     </row>
-    <row r="20" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="5" t="s">
         <v>17</v>
@@ -1760,7 +1760,7 @@
       <c r="W20" s="5"/>
       <c r="X20" s="5"/>
     </row>
-    <row r="21" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="5" t="s">
         <v>38</v>
@@ -1796,7 +1796,7 @@
       <c r="W21" s="5"/>
       <c r="X21" s="5"/>
     </row>
-    <row r="22" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="5" t="s">
         <v>27</v>
@@ -1824,7 +1824,7 @@
       <c r="W22" s="2"/>
       <c r="X22" s="2"/>
     </row>
-    <row r="23" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="4" t="s">
         <v>40</v>
@@ -1852,7 +1852,7 @@
       <c r="W23" s="4"/>
       <c r="X23" s="4"/>
     </row>
-    <row r="24" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="8" t="s">
         <v>41</v>
@@ -1880,7 +1880,7 @@
       <c r="W24" s="8"/>
       <c r="X24" s="8"/>
     </row>
-    <row r="25" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="5" t="s">
         <v>42</v>
@@ -1910,7 +1910,7 @@
       <c r="W25" s="5"/>
       <c r="X25" s="5"/>
     </row>
-    <row r="26" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="5" t="s">
         <v>44</v>
@@ -1938,10 +1938,10 @@
       <c r="W26" s="5"/>
       <c r="X26" s="2"/>
     </row>
-    <row r="27" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="15" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -1966,7 +1966,7 @@
       <c r="W27" s="5"/>
       <c r="X27" s="5"/>
     </row>
-    <row r="28" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1994,7 +1994,7 @@
       <c r="W28" s="5"/>
       <c r="X28" s="5"/>
     </row>
-    <row r="29" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="5" t="s">
         <v>46</v>
@@ -2024,7 +2024,7 @@
       <c r="W29" s="12"/>
       <c r="X29" s="12"/>
     </row>
-    <row r="30" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="5" t="s">
         <v>48</v>
@@ -2054,7 +2054,7 @@
       <c r="W30" s="5"/>
       <c r="X30" s="5"/>
     </row>
-    <row r="31" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="5" t="s">
         <v>50</v>
@@ -2082,7 +2082,7 @@
       <c r="W31" s="5"/>
       <c r="X31" s="5"/>
     </row>
-    <row r="32" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="8" t="s">
         <v>51</v>
@@ -2110,7 +2110,7 @@
       <c r="W32" s="8"/>
       <c r="X32" s="8"/>
     </row>
-    <row r="33" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -2138,7 +2138,7 @@
       <c r="W33" s="5"/>
       <c r="X33" s="5"/>
     </row>
-    <row r="34" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="5" t="s">
         <v>53</v>
@@ -2166,7 +2166,7 @@
       <c r="W34" s="5"/>
       <c r="X34" s="5"/>
     </row>
-    <row r="35" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="5" t="s">
         <v>54</v>
@@ -2194,7 +2194,7 @@
       <c r="W35" s="5"/>
       <c r="X35" s="5"/>
     </row>
-    <row r="36" spans="1:24" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:24" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -2220,7 +2220,7 @@
       <c r="W36" s="2"/>
       <c r="X36" s="2"/>
     </row>
-    <row r="37" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="8" t="s">
         <v>55</v>
@@ -2248,7 +2248,7 @@
       <c r="W37" s="8"/>
       <c r="X37" s="8"/>
     </row>
-    <row r="38" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="9" t="s">
         <v>56</v>
@@ -2276,7 +2276,7 @@
       <c r="W38" s="9"/>
       <c r="X38" s="9"/>
     </row>
-    <row r="39" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="8" t="s">
         <v>57</v>
@@ -2306,7 +2306,7 @@
       <c r="W39" s="12"/>
       <c r="X39" s="12"/>
     </row>
-    <row r="40" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="13" t="s">
         <v>59</v>
@@ -2334,7 +2334,7 @@
       <c r="W40" s="14"/>
       <c r="X40" s="14"/>
     </row>
-    <row r="41" spans="1:24" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:24" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2360,7 +2360,7 @@
       <c r="W41" s="2"/>
       <c r="X41" s="2"/>
     </row>
-    <row r="42" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="8" t="s">
         <v>60</v>
@@ -2390,7 +2390,7 @@
       <c r="W42" s="5"/>
       <c r="X42" s="5"/>
     </row>
-    <row r="43" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="5" t="s">
         <v>62</v>
@@ -2418,7 +2418,7 @@
       <c r="W43" s="5"/>
       <c r="X43" s="5"/>
     </row>
-    <row r="44" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="5" t="s">
         <v>63</v>
@@ -2446,7 +2446,7 @@
       <c r="W44" s="5"/>
       <c r="X44" s="5"/>
     </row>
-    <row r="45" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="8" t="s">
         <v>64</v>
@@ -2474,7 +2474,7 @@
       <c r="W45" s="2"/>
       <c r="X45" s="2"/>
     </row>
-    <row r="46" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="8" t="s">
         <v>65</v>
@@ -2502,7 +2502,7 @@
       <c r="W46" s="8"/>
       <c r="X46" s="8"/>
     </row>
-    <row r="47" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="5" t="s">
         <v>66</v>
@@ -2530,7 +2530,7 @@
       <c r="W47" s="5"/>
       <c r="X47" s="5"/>
     </row>
-    <row r="48" spans="1:24" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:24" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="11" t="s">
         <v>67</v>
@@ -2558,7 +2558,7 @@
       <c r="W48" s="5"/>
       <c r="X48" s="5"/>
     </row>
-    <row r="49" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="8" t="s">
         <v>68</v>
@@ -2588,7 +2588,7 @@
       <c r="W49" s="5"/>
       <c r="X49" s="5"/>
     </row>
-    <row r="50" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="5" t="s">
         <v>70</v>
@@ -2616,7 +2616,7 @@
       <c r="W50" s="5"/>
       <c r="X50" s="2"/>
     </row>
-    <row r="51" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="8" t="s">
         <v>71</v>
@@ -2644,7 +2644,7 @@
       <c r="W51" s="2"/>
       <c r="X51" s="2"/>
     </row>
-    <row r="52" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="5" t="s">
         <v>72</v>
@@ -2672,7 +2672,7 @@
       <c r="W52" s="5"/>
       <c r="X52" s="5"/>
     </row>
-    <row r="53" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="5" t="s">
         <v>73</v>
@@ -2700,7 +2700,7 @@
       <c r="W53" s="5"/>
       <c r="X53" s="5"/>
     </row>
-    <row r="54" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="8" t="s">
         <v>74</v>
@@ -2728,7 +2728,7 @@
       <c r="W54" s="2"/>
       <c r="X54" s="2"/>
     </row>
-    <row r="55" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="5" t="s">
         <v>75</v>
@@ -2756,7 +2756,7 @@
       <c r="W55" s="5"/>
       <c r="X55" s="5"/>
     </row>
-    <row r="56" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="5" t="s">
         <v>76</v>
@@ -2784,7 +2784,7 @@
       <c r="W56" s="5"/>
       <c r="X56" s="5"/>
     </row>
-    <row r="57" spans="1:24" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:24" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="5" t="s">
         <v>77</v>
@@ -2812,7 +2812,7 @@
       <c r="W57" s="5"/>
       <c r="X57" s="5"/>
     </row>
-    <row r="58" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="8" t="s">
         <v>78</v>
@@ -2840,7 +2840,7 @@
       <c r="W58" s="8"/>
       <c r="X58" s="8"/>
     </row>
-    <row r="59" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="5" t="s">
         <v>79</v>
@@ -2868,7 +2868,7 @@
       <c r="W59" s="5"/>
       <c r="X59" s="5"/>
     </row>
-    <row r="60" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="5" t="s">
         <v>80</v>
@@ -2896,7 +2896,7 @@
       <c r="W60" s="5"/>
       <c r="X60" s="5"/>
     </row>
-    <row r="61" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="5" t="s">
         <v>81</v>
@@ -2924,7 +2924,7 @@
       <c r="W61" s="5"/>
       <c r="X61" s="5"/>
     </row>
-    <row r="62" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="5" t="s">
         <v>82</v>
@@ -2952,7 +2952,7 @@
       <c r="W62" s="5"/>
       <c r="X62" s="5"/>
     </row>
-    <row r="63" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="B63" s="8" t="s">
         <v>83</v>
@@ -2980,7 +2980,7 @@
       <c r="W63" s="8"/>
       <c r="X63" s="8"/>
     </row>
-    <row r="64" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="B64" s="5" t="s">
         <v>84</v>
@@ -3008,7 +3008,7 @@
       <c r="W64" s="5"/>
       <c r="X64" s="5"/>
     </row>
-    <row r="65" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="10" t="s">
         <v>85</v>
@@ -3036,7 +3036,7 @@
       <c r="W65" s="8"/>
       <c r="X65" s="8"/>
     </row>
-    <row r="66" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="8" t="s">
         <v>86</v>
@@ -3064,7 +3064,7 @@
       <c r="W66" s="8"/>
       <c r="X66" s="8"/>
     </row>
-    <row r="67" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="5" t="s">
         <v>87</v>
@@ -3092,7 +3092,7 @@
       <c r="W67" s="5"/>
       <c r="X67" s="5"/>
     </row>
-    <row r="68" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="5" t="s">
         <v>154</v>
@@ -3120,7 +3120,7 @@
       <c r="W68" s="5"/>
       <c r="X68" s="5"/>
     </row>
-    <row r="69" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="8" t="s">
         <v>88</v>
@@ -3148,7 +3148,7 @@
       <c r="W69" s="8"/>
       <c r="X69" s="8"/>
     </row>
-    <row r="70" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="5" t="s">
         <v>89</v>
@@ -3176,7 +3176,7 @@
       <c r="W70" s="5"/>
       <c r="X70" s="5"/>
     </row>
-    <row r="71" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="8" t="s">
         <v>153</v>
@@ -3204,7 +3204,7 @@
       <c r="W71" s="8"/>
       <c r="X71" s="8"/>
     </row>
-    <row r="72" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
       <c r="B72" s="8" t="s">
         <v>90</v>
@@ -3232,7 +3232,7 @@
       <c r="W72" s="8"/>
       <c r="X72" s="8"/>
     </row>
-    <row r="73" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
       <c r="B73" s="5" t="s">
         <v>91</v>
@@ -3260,7 +3260,7 @@
       <c r="W73" s="5"/>
       <c r="X73" s="5"/>
     </row>
-    <row r="74" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="5" t="s">
         <v>92</v>
@@ -3288,7 +3288,7 @@
       <c r="W74" s="5"/>
       <c r="X74" s="5"/>
     </row>
-    <row r="75" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
       <c r="B75" s="5" t="s">
         <v>93</v>
@@ -3316,7 +3316,7 @@
       <c r="W75" s="5"/>
       <c r="X75" s="5"/>
     </row>
-    <row r="76" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="5" t="s">
         <v>94</v>
@@ -3344,7 +3344,7 @@
       <c r="W76" s="5"/>
       <c r="X76" s="2"/>
     </row>
-    <row r="77" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
       <c r="B77" s="5" t="s">
         <v>95</v>
@@ -3372,7 +3372,7 @@
       <c r="W77" s="5"/>
       <c r="X77" s="5"/>
     </row>
-    <row r="78" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="5" t="s">
         <v>96</v>
@@ -3400,7 +3400,7 @@
       <c r="W78" s="5"/>
       <c r="X78" s="5"/>
     </row>
-    <row r="79" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
       <c r="B79" s="5" t="s">
         <v>97</v>
@@ -3428,7 +3428,7 @@
       <c r="W79" s="5"/>
       <c r="X79" s="5"/>
     </row>
-    <row r="80" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="5" t="s">
         <v>98</v>
@@ -3456,7 +3456,7 @@
       <c r="W80" s="5"/>
       <c r="X80" s="5"/>
     </row>
-    <row r="81" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="5" t="s">
         <v>99</v>
@@ -3484,7 +3484,7 @@
       <c r="W81" s="5"/>
       <c r="X81" s="5"/>
     </row>
-    <row r="82" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
       <c r="B82" s="9" t="s">
         <v>100</v>
@@ -3512,7 +3512,7 @@
       <c r="W82" s="9"/>
       <c r="X82" s="9"/>
     </row>
-    <row r="83" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="5" t="s">
         <v>101</v>
@@ -3540,7 +3540,7 @@
       <c r="W83" s="5"/>
       <c r="X83" s="5"/>
     </row>
-    <row r="84" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
       <c r="B84" s="5" t="s">
         <v>102</v>
@@ -3568,7 +3568,7 @@
       <c r="W84" s="5"/>
       <c r="X84" s="5"/>
     </row>
-    <row r="85" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
       <c r="B85" s="5" t="s">
         <v>103</v>
@@ -3596,7 +3596,7 @@
       <c r="W85" s="5"/>
       <c r="X85" s="5"/>
     </row>
-    <row r="86" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
       <c r="B86" s="5" t="s">
         <v>104</v>
@@ -3624,7 +3624,7 @@
       <c r="W86" s="5"/>
       <c r="X86" s="5"/>
     </row>
-    <row r="87" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
       <c r="B87" s="5" t="s">
         <v>105</v>
@@ -3652,7 +3652,7 @@
       <c r="W87" s="5"/>
       <c r="X87" s="5"/>
     </row>
-    <row r="88" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
       <c r="B88" s="5" t="s">
         <v>106</v>
@@ -3680,7 +3680,7 @@
       <c r="W88" s="5"/>
       <c r="X88" s="5"/>
     </row>
-    <row r="89" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
       <c r="B89" s="5" t="s">
         <v>107</v>
@@ -3708,7 +3708,7 @@
       <c r="W89" s="5"/>
       <c r="X89" s="5"/>
     </row>
-    <row r="90" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
       <c r="B90" s="5" t="s">
         <v>108</v>
@@ -3736,7 +3736,7 @@
       <c r="W90" s="5"/>
       <c r="X90" s="5"/>
     </row>
-    <row r="91" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
       <c r="B91" s="5" t="s">
         <v>109</v>
@@ -3764,7 +3764,7 @@
       <c r="W91" s="5"/>
       <c r="X91" s="5"/>
     </row>
-    <row r="92" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
       <c r="B92" s="5" t="s">
         <v>110</v>
@@ -3792,7 +3792,7 @@
       <c r="W92" s="5"/>
       <c r="X92" s="5"/>
     </row>
-    <row r="93" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
       <c r="B93" s="5" t="s">
         <v>111</v>
@@ -3820,7 +3820,7 @@
       <c r="W93" s="5"/>
       <c r="X93" s="5"/>
     </row>
-    <row r="94" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
       <c r="B94" s="5" t="s">
         <v>112</v>
@@ -3848,7 +3848,7 @@
       <c r="W94" s="5"/>
       <c r="X94" s="5"/>
     </row>
-    <row r="95" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
       <c r="B95" s="5" t="s">
         <v>113</v>
@@ -3876,7 +3876,7 @@
       <c r="W95" s="5"/>
       <c r="X95" s="5"/>
     </row>
-    <row r="96" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="5" t="s">
         <v>114</v>
@@ -3904,7 +3904,7 @@
       <c r="W96" s="5"/>
       <c r="X96" s="5"/>
     </row>
-    <row r="97" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="5" t="s">
         <v>115</v>
@@ -3932,7 +3932,7 @@
       <c r="W97" s="5"/>
       <c r="X97" s="5"/>
     </row>
-    <row r="98" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="5" t="s">
         <v>116</v>
@@ -3960,7 +3960,7 @@
       <c r="W98" s="5"/>
       <c r="X98" s="5"/>
     </row>
-    <row r="99" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="5" t="s">
         <v>117</v>
@@ -3988,7 +3988,7 @@
       <c r="W99" s="5"/>
       <c r="X99" s="5"/>
     </row>
-    <row r="100" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="5" t="s">
         <v>118</v>
@@ -4016,7 +4016,7 @@
       <c r="W100" s="5"/>
       <c r="X100" s="5"/>
     </row>
-    <row r="101" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="5" t="s">
         <v>119</v>
@@ -4044,7 +4044,7 @@
       <c r="W101" s="5"/>
       <c r="X101" s="5"/>
     </row>
-    <row r="102" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="5" t="s">
         <v>120</v>
@@ -4072,7 +4072,7 @@
       <c r="W102" s="5"/>
       <c r="X102" s="5"/>
     </row>
-    <row r="103" spans="1:24" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:24" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -4098,7 +4098,7 @@
       <c r="W103" s="2"/>
       <c r="X103" s="2"/>
     </row>
-    <row r="104" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="8" t="s">
         <v>121</v>
@@ -4126,7 +4126,7 @@
       <c r="W104" s="8"/>
       <c r="X104" s="8"/>
     </row>
-    <row r="105" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="8" t="s">
         <v>122</v>
@@ -4154,7 +4154,7 @@
       <c r="W105" s="8"/>
       <c r="X105" s="8"/>
     </row>
-    <row r="106" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="5" t="s">
         <v>123</v>
@@ -4182,7 +4182,7 @@
       <c r="W106" s="5"/>
       <c r="X106" s="5"/>
     </row>
-    <row r="107" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="5" t="s">
         <v>124</v>
@@ -4210,7 +4210,7 @@
       <c r="W107" s="5"/>
       <c r="X107" s="5"/>
     </row>
-    <row r="108" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="5" t="s">
         <v>125</v>
@@ -4238,7 +4238,7 @@
       <c r="W108" s="5"/>
       <c r="X108" s="5"/>
     </row>
-    <row r="109" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="5" t="s">
         <v>126</v>
@@ -4266,7 +4266,7 @@
       <c r="W109" s="5"/>
       <c r="X109" s="5"/>
     </row>
-    <row r="110" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="5" t="s">
         <v>127</v>
@@ -4294,7 +4294,7 @@
       <c r="W110" s="5"/>
       <c r="X110" s="5"/>
     </row>
-    <row r="111" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="8" t="s">
         <v>128</v>
@@ -4322,7 +4322,7 @@
       <c r="W111" s="8"/>
       <c r="X111" s="8"/>
     </row>
-    <row r="112" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
       <c r="B112" s="5" t="s">
         <v>129</v>
@@ -4350,7 +4350,7 @@
       <c r="W112" s="5"/>
       <c r="X112" s="5"/>
     </row>
-    <row r="113" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="5" t="s">
         <v>130</v>
@@ -4378,7 +4378,7 @@
       <c r="W113" s="5"/>
       <c r="X113" s="5"/>
     </row>
-    <row r="114" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
       <c r="B114" s="5" t="s">
         <v>131</v>
@@ -4406,7 +4406,7 @@
       <c r="W114" s="5"/>
       <c r="X114" s="5"/>
     </row>
-    <row r="115" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
       <c r="B115" s="5" t="s">
         <v>132</v>
@@ -4434,7 +4434,7 @@
       <c r="W115" s="5"/>
       <c r="X115" s="5"/>
     </row>
-    <row r="116" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
       <c r="B116" s="8" t="s">
         <v>133</v>
@@ -4462,7 +4462,7 @@
       <c r="W116" s="8"/>
       <c r="X116" s="8"/>
     </row>
-    <row r="117" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
       <c r="B117" s="5" t="s">
         <v>134</v>
@@ -4490,7 +4490,7 @@
       <c r="W117" s="5"/>
       <c r="X117" s="5"/>
     </row>
-    <row r="118" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2"/>
       <c r="B118" s="5" t="s">
         <v>135</v>
@@ -4518,7 +4518,7 @@
       <c r="W118" s="5"/>
       <c r="X118" s="5"/>
     </row>
-    <row r="119" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2"/>
       <c r="B119" s="5" t="s">
         <v>136</v>
@@ -4546,7 +4546,7 @@
       <c r="W119" s="5"/>
       <c r="X119" s="5"/>
     </row>
-    <row r="120" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2"/>
       <c r="B120" s="5" t="s">
         <v>137</v>
@@ -4574,7 +4574,7 @@
       <c r="W120" s="5"/>
       <c r="X120" s="5"/>
     </row>
-    <row r="121" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2"/>
       <c r="B121" s="5" t="s">
         <v>138</v>
@@ -4602,7 +4602,7 @@
       <c r="W121" s="5"/>
       <c r="X121" s="5"/>
     </row>
-    <row r="122" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2"/>
       <c r="B122" s="5" t="s">
         <v>139</v>
@@ -4630,7 +4630,7 @@
       <c r="W122" s="5"/>
       <c r="X122" s="5"/>
     </row>
-    <row r="123" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2"/>
       <c r="B123" s="8" t="s">
         <v>140</v>
@@ -4658,7 +4658,7 @@
       <c r="W123" s="8"/>
       <c r="X123" s="8"/>
     </row>
-    <row r="124" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2"/>
       <c r="B124" s="5" t="s">
         <v>141</v>
@@ -4686,7 +4686,7 @@
       <c r="W124" s="5"/>
       <c r="X124" s="5"/>
     </row>
-    <row r="125" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2"/>
       <c r="B125" s="5" t="s">
         <v>142</v>
@@ -4714,7 +4714,7 @@
       <c r="W125" s="5"/>
       <c r="X125" s="5"/>
     </row>
-    <row r="126" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2"/>
       <c r="B126" s="5" t="s">
         <v>143</v>
@@ -4742,7 +4742,7 @@
       <c r="W126" s="5"/>
       <c r="X126" s="5"/>
     </row>
-    <row r="127" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2"/>
       <c r="B127" s="5" t="s">
         <v>144</v>
@@ -4770,7 +4770,7 @@
       <c r="W127" s="5"/>
       <c r="X127" s="5"/>
     </row>
-    <row r="128" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="5" t="s">
         <v>145</v>
@@ -4798,7 +4798,7 @@
       <c r="W128" s="5"/>
       <c r="X128" s="5"/>
     </row>
-    <row r="129" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2"/>
       <c r="B129" s="6" t="s">
         <v>146</v>
@@ -4828,7 +4828,7 @@
       <c r="W129" s="6"/>
       <c r="X129" s="6"/>
     </row>
-    <row r="130" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
       <c r="B130" s="7" t="s">
         <v>148</v>
@@ -4856,7 +4856,7 @@
       <c r="W130" s="7"/>
       <c r="X130" s="7"/>
     </row>
-    <row r="131" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -4882,7 +4882,7 @@
       <c r="W131" s="2"/>
       <c r="X131" s="2"/>
     </row>
-    <row r="132" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -4908,7 +4908,7 @@
       <c r="W132" s="2"/>
       <c r="X132" s="2"/>
     </row>
-    <row r="133" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -4934,7 +4934,7 @@
       <c r="W133" s="2"/>
       <c r="X133" s="2"/>
     </row>
-    <row r="134" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -4960,7 +4960,7 @@
       <c r="W134" s="2"/>
       <c r="X134" s="2"/>
     </row>
-    <row r="135" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -4990,7 +4990,7 @@
       <c r="W135" s="5"/>
       <c r="X135" s="5"/>
     </row>
-    <row r="136" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -5018,7 +5018,7 @@
       <c r="W136" s="5"/>
       <c r="X136" s="2"/>
     </row>
-    <row r="137" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -5048,7 +5048,7 @@
       <c r="W137" s="2"/>
       <c r="X137" s="2"/>
     </row>
-    <row r="138" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>

</xml_diff>